<commit_message>
Add calendar-day footnote from original sheet to printable schedule
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GrqacRrrxsErzucVfyVZnY
</commit_message>
<xml_diff>
--- a/Pownal Security Schedule.xlsx
+++ b/Pownal Security Schedule.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Security Schedule" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Security Schedule'!$A$1:$K$24</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Security Schedule'!$A$1:$K$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +48,10 @@
     <font>
       <b val="1"/>
       <sz val="9.5"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="7">
@@ -109,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -129,6 +133,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -494,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -898,8 +905,16 @@
       <c r="C23" s="8" t="n"/>
     </row>
     <row r="24" ht="10" customHeight="1"/>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Please note that shifts are organized by calendar day. Even if a shift extends into the early morning hours, it is recorded under the day it begins to maintain scheduling consistency.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
+    <mergeCell ref="A25:K25"/>
     <mergeCell ref="I9:K9"/>
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="A9:C9"/>

</xml_diff>

<commit_message>
Switch schedule to portrait layout with days stacked vertically
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GrqacRrrxsErzucVfyVZnY
</commit_message>
<xml_diff>
--- a/Pownal Security Schedule.xlsx
+++ b/Pownal Security Schedule.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Security Schedule" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Security Schedule'!$A$1:$K$25</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Security Schedule'!$A$1:$C$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,21 +33,21 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00000000"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="9.5"/>
     </font>
     <font>
       <i val="1"/>
@@ -122,13 +122,13 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -501,23 +501,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="1.5" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="1.5" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
+    <col width="37" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>POWNAL SECURITY SCHEDULE</t>
@@ -525,87 +517,35 @@
       </c>
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="6" customHeight="1"/>
-    <row r="3" ht="22" customHeight="1">
+    </row>
+    <row r="2" ht="5" customHeight="1"/>
+    <row r="3" ht="18" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Volunteer 1</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Volunteer 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
           <t>August 11th  TUESDAY</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>August 12th  WEDNESDAY</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>August 13th  THURSDAY</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="n"/>
-      <c r="K3" s="4" t="n"/>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Shift</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Volunteer 1</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Volunteer 2</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Shift</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Volunteer 1</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Volunteer 2</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>Shift</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>Volunteer 1</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
-          <t>Volunteer 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1">
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
           <t>5pm - 10pm</t>
@@ -613,22 +553,8 @@
       </c>
       <c r="B5" s="8" t="n"/>
       <c r="C5" s="8" t="n"/>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>5pm - 10pm</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
-      <c r="I5" s="7" t="inlineStr">
-        <is>
-          <t>5pm - 10pm</t>
-        </is>
-      </c>
-      <c r="J5" s="8" t="n"/>
-      <c r="K5" s="8" t="n"/>
-    </row>
-    <row r="6" ht="42" customHeight="1">
+    </row>
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>10pm - 3am</t>
@@ -636,22 +562,8 @@
       </c>
       <c r="B6" s="8" t="n"/>
       <c r="C6" s="8" t="n"/>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>10pm - 3am</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
-      <c r="I6" s="7" t="inlineStr">
-        <is>
-          <t>10pm - 3am</t>
-        </is>
-      </c>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="8" t="n"/>
-    </row>
-    <row r="7" ht="42" customHeight="1">
+    </row>
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>3am - 8am (when volunteers arrive)</t>
@@ -659,225 +571,125 @@
       </c>
       <c r="B7" s="8" t="n"/>
       <c r="C7" s="8" t="n"/>
-      <c r="E7" s="7" t="inlineStr">
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>August 12th  WEDNESDAY</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>5pm - 10pm</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>10pm - 3am</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>3am - 8am (when volunteers arrive)</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>3am - 8am (when volunteers arrive)</t>
-        </is>
-      </c>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="8" t="n"/>
-    </row>
-    <row r="8" ht="10" customHeight="1"/>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>August 14th  FRIDAY</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>August 15th  SATURDAY</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="4" t="n"/>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>August 16th  SUNDAY</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="n"/>
-      <c r="K9" s="4" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Shift</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Volunteer 1</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Volunteer 2</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Shift</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Volunteer 1</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Volunteer 2</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>Shift</t>
-        </is>
-      </c>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>Volunteer 1</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
-          <t>Volunteer 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>5pm - 10pm</t>
         </is>
       </c>
       <c r="B11" s="8" t="n"/>
       <c r="C11" s="8" t="n"/>
-      <c r="E11" s="7" t="inlineStr">
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>August 13th  THURSDAY</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>5pm - 10pm</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="n"/>
-      <c r="G11" s="8" t="n"/>
-      <c r="I11" s="7" t="inlineStr">
-        <is>
-          <t>7am - 12pm</t>
-        </is>
-      </c>
-      <c r="J11" s="8" t="n"/>
-      <c r="K11" s="8" t="n"/>
-    </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>10pm - 3am</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="n"/>
-      <c r="C12" s="8" t="n"/>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>10pm - 3am</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="n"/>
-      <c r="G12" s="8" t="n"/>
-      <c r="I12" s="7" t="inlineStr">
-        <is>
-          <t>12pm - 5pm</t>
-        </is>
-      </c>
-      <c r="J12" s="8" t="n"/>
-      <c r="K12" s="8" t="n"/>
-    </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>3am - 8am (when volunteers arrive)</t>
         </is>
       </c>
       <c r="B13" s="8" t="n"/>
       <c r="C13" s="8" t="n"/>
-      <c r="E13" s="7" t="inlineStr">
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>10pm - 3am</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>3am - 8am (when volunteers arrive)</t>
         </is>
       </c>
-      <c r="F13" s="8" t="n"/>
-      <c r="G13" s="8" t="n"/>
-      <c r="I13" s="7" t="inlineStr">
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="8" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>August 14th  FRIDAY</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>5pm - 10pm</t>
         </is>
       </c>
-      <c r="J13" s="8" t="n"/>
-      <c r="K13" s="8" t="n"/>
-    </row>
-    <row r="14" ht="42" customHeight="1">
-      <c r="I14" s="7" t="inlineStr">
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>10pm - 3am</t>
         </is>
       </c>
-      <c r="J14" s="8" t="n"/>
-      <c r="K14" s="8" t="n"/>
-    </row>
-    <row r="15" ht="42" customHeight="1">
-      <c r="I15" s="7" t="inlineStr">
-        <is>
-          <t>3am - 8am</t>
-        </is>
-      </c>
-      <c r="J15" s="8" t="n"/>
-      <c r="K15" s="8" t="n"/>
-    </row>
-    <row r="16" ht="10" customHeight="1"/>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>August 17th  MONDAY</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="4" t="n"/>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Shift</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Volunteer 1</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Volunteer 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="42" customHeight="1">
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="8" t="n"/>
+    </row>
+    <row r="19" ht="36" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>7am - 12pm</t>
+          <t>3am - 8am (when volunteers arrive)</t>
         </is>
       </c>
       <c r="B19" s="8" t="n"/>
       <c r="C19" s="8" t="n"/>
     </row>
-    <row r="20" ht="42" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>12pm - 5pm</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="8" t="n"/>
-    </row>
-    <row r="21" ht="42" customHeight="1">
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>August 15th  SATURDAY</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="36" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
           <t>5pm - 10pm</t>
@@ -886,7 +698,7 @@
       <c r="B21" s="8" t="n"/>
       <c r="C21" s="8" t="n"/>
     </row>
-    <row r="22" ht="42" customHeight="1">
+    <row r="22" ht="36" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
         <is>
           <t>10pm - 3am</t>
@@ -895,7 +707,7 @@
       <c r="B22" s="8" t="n"/>
       <c r="C22" s="8" t="n"/>
     </row>
-    <row r="23" ht="42" customHeight="1">
+    <row r="23" ht="36" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
         <is>
           <t>3am - 8am (when volunteers arrive)</t>
@@ -904,9 +716,116 @@
       <c r="B23" s="8" t="n"/>
       <c r="C23" s="8" t="n"/>
     </row>
-    <row r="24" ht="10" customHeight="1"/>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>August 16th  SUNDAY</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>7am - 12pm</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>12pm - 5pm</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="8" t="n"/>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>5pm - 10pm</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="8" t="n"/>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>10pm - 3am</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="8" t="n"/>
+    </row>
+    <row r="29" ht="36" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>3am - 8am</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="8" t="n"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>August 17th  MONDAY</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="n"/>
+      <c r="C30" s="6" t="n"/>
+    </row>
+    <row r="31" ht="36" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>7am - 12pm</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="8" t="n"/>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>12pm - 5pm</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="8" t="n"/>
+    </row>
+    <row r="33" ht="36" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>5pm - 10pm</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+    </row>
+    <row r="34" ht="36" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>10pm - 3am</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="8" t="n"/>
+    </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>3am - 8am (when volunteers arrive)</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="n"/>
+      <c r="C35" s="8" t="n"/>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="9" t="inlineStr">
         <is>
           <t>Please note that shifts are organized by calendar day. Even if a shift extends into the early morning hours, it is recorded under the day it begins to maintain scheduling consistency.</t>
         </is>
@@ -914,17 +833,17 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A25:K25"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="I3:K3"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="1" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>